<commit_message>
Painel: sem lote registrado, a coluna de melhor % fica vazia
Li a planilha ja convertida no Drive e as 16 linhas mostravam "0,0%" em
"Melhor % bruto" sem nenhum lote lancado: MAX de um intervalo vazio
devolve zero, e zero ali se le como "fiz e zerei", nao como "ainda nao
fiz". Agora a celula so mostra numero quando existe lote.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PtPAoX2xeve2DccJV9EvXQ
</commit_message>
<xml_diff>
--- a/src/data/squads-md/tcdf-concurso/planilha/TCDF-acompanhamento.xlsx
+++ b/src/data/squads-md/tcdf-concurso/planilha/TCDF-acompanhamento.xlsx
@@ -675,7 +675,7 @@
         <v/>
       </c>
       <c r="G5" s="6">
-        <f>IFERROR(MAX('AFO'!F49:F68),"")</f>
+        <f>IF(COUNT('AFO'!C49:C68)=0,"",MAX('AFO'!F49:F68))</f>
         <v/>
       </c>
       <c r="H5" s="6">
@@ -709,7 +709,7 @@
         <v/>
       </c>
       <c r="G6" s="6">
-        <f>IFERROR(MAX('D. Tributário'!F29:F48),"")</f>
+        <f>IF(COUNT('D. Tributário'!C29:C48)=0,"",MAX('D. Tributário'!F29:F48))</f>
         <v/>
       </c>
       <c r="H6" s="6">
@@ -743,7 +743,7 @@
         <v/>
       </c>
       <c r="G7" s="6">
-        <f>IFERROR(MAX('D. Administrativo'!F68:F87),"")</f>
+        <f>IF(COUNT('D. Administrativo'!C68:C87)=0,"",MAX('D. Administrativo'!F68:F87))</f>
         <v/>
       </c>
       <c r="H7" s="6">
@@ -777,7 +777,7 @@
         <v/>
       </c>
       <c r="G8" s="6">
-        <f>IFERROR(MAX('Gestão de Contratos'!F25:F44),"")</f>
+        <f>IF(COUNT('Gestão de Contratos'!C25:C44)=0,"",MAX('Gestão de Contratos'!F25:F44))</f>
         <v/>
       </c>
       <c r="H8" s="6">
@@ -811,7 +811,7 @@
         <v/>
       </c>
       <c r="G9" s="6">
-        <f>IFERROR(MAX('D. Constitucional'!F40:F59),"")</f>
+        <f>IF(COUNT('D. Constitucional'!C40:C59)=0,"",MAX('D. Constitucional'!F40:F59))</f>
         <v/>
       </c>
       <c r="H9" s="6">
@@ -845,7 +845,7 @@
         <v/>
       </c>
       <c r="G10" s="6">
-        <f>IFERROR(MAX('LO e RI do TCDF'!F24:F43),"")</f>
+        <f>IF(COUNT('LO e RI do TCDF'!C24:C43)=0,"",MAX('LO e RI do TCDF'!F24:F43))</f>
         <v/>
       </c>
       <c r="H10" s="6">
@@ -879,7 +879,7 @@
         <v/>
       </c>
       <c r="G11" s="6">
-        <f>IFERROR(MAX('LODF'!F18:F37),"")</f>
+        <f>IF(COUNT('LODF'!C18:C37)=0,"",MAX('LODF'!F18:F37))</f>
         <v/>
       </c>
       <c r="H11" s="6">
@@ -913,7 +913,7 @@
         <v/>
       </c>
       <c r="G12" s="6">
-        <f>IFERROR(MAX('Adm. Geral e Pública'!F48:F67),"")</f>
+        <f>IF(COUNT('Adm. Geral e Pública'!C48:C67)=0,"",MAX('Adm. Geral e Pública'!F48:F67))</f>
         <v/>
       </c>
       <c r="H12" s="6">
@@ -947,7 +947,7 @@
         <v/>
       </c>
       <c r="G13" s="6">
-        <f>IFERROR(MAX('Análise de Dados'!F31:F50),"")</f>
+        <f>IF(COUNT('Análise de Dados'!C31:C50)=0,"",MAX('Análise de Dados'!F31:F50))</f>
         <v/>
       </c>
       <c r="H13" s="6">
@@ -981,7 +981,7 @@
         <v/>
       </c>
       <c r="G14" s="6">
-        <f>IFERROR(MAX('LC 840 Servidores'!F21:F40),"")</f>
+        <f>IF(COUNT('LC 840 Servidores'!C21:C40)=0,"",MAX('LC 840 Servidores'!F21:F40))</f>
         <v/>
       </c>
       <c r="H14" s="6">
@@ -1015,7 +1015,7 @@
         <v/>
       </c>
       <c r="G15" s="6">
-        <f>IFERROR(MAX('D. Previdenciário'!F20:F39),"")</f>
+        <f>IF(COUNT('D. Previdenciário'!C20:C39)=0,"",MAX('D. Previdenciário'!F20:F39))</f>
         <v/>
       </c>
       <c r="H15" s="6">
@@ -1049,7 +1049,7 @@
         <v/>
       </c>
       <c r="G16" s="6">
-        <f>IFERROR(MAX('D. Civil'!F23:F42),"")</f>
+        <f>IF(COUNT('D. Civil'!C23:C42)=0,"",MAX('D. Civil'!F23:F42))</f>
         <v/>
       </c>
       <c r="H16" s="6">
@@ -1083,7 +1083,7 @@
         <v/>
       </c>
       <c r="G17" s="6">
-        <f>IFERROR(MAX('Português'!F33:F52),"")</f>
+        <f>IF(COUNT('Português'!C33:C52)=0,"",MAX('Português'!F33:F52))</f>
         <v/>
       </c>
       <c r="H17" s="6">
@@ -1117,7 +1117,7 @@
         <v/>
       </c>
       <c r="G18" s="6">
-        <f>IFERROR(MAX('RLM'!F27:F46),"")</f>
+        <f>IF(COUNT('RLM'!C27:C46)=0,"",MAX('RLM'!F27:F46))</f>
         <v/>
       </c>
       <c r="H18" s="6">
@@ -1151,7 +1151,7 @@
         <v/>
       </c>
       <c r="G19" s="6">
-        <f>IFERROR(MAX('DF e Mulheres'!F16:F35),"")</f>
+        <f>IF(COUNT('DF e Mulheres'!C16:C35)=0,"",MAX('DF e Mulheres'!F16:F35))</f>
         <v/>
       </c>
       <c r="H19" s="6">
@@ -1185,7 +1185,7 @@
         <v/>
       </c>
       <c r="G20" s="6">
-        <f>IFERROR(MAX('Primeiros Socorros'!F23:F42),"")</f>
+        <f>IF(COUNT('Primeiros Socorros'!C23:C42)=0,"",MAX('Primeiros Socorros'!F23:F42))</f>
         <v/>
       </c>
       <c r="H20" s="6">

</xml_diff>